<commit_message>
feat(backend/data): add 100-patient synthetic dataset and ingestion pipeline
- seed_dev.py: full rewrite — seeds 100 patients with realistic clinical
  profiles (diagnoses, medications, labs, allergies, timeline events)
- generate_100_patients.py: deterministic patient generator using Faker
  with Vietnamese name support; outputs patients_100.xlsx
- ingest_synthetic_dataset.py: new script to batch-ingest patient PDFs,
  drug formularies, and clinical guidelines into the vector store
- import_patients_seed.py: helper to bulk-import from xlsx to DB
- inspect_patients.py: diagnostic script to verify seed data integrity
- data/: add synthetic dataset folders (drugs, guidelines, patient docs,
  labs, metadata, security audit logs for 100 patients)
- tests: add test_observability.py; extend test_chat_endpoint and
  test_retrieval_sql for new retrieval and 100-patient data paths
</commit_message>
<xml_diff>
--- a/app/backend/data/patients_100.xlsx
+++ b/app/backend/data/patients_100.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Võ Quang Hùng</t>
+          <t>Vo Quang Hung</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lê Ngọc Hạnh</t>
+          <t>Le Ngoc Hanh</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Võ Văn Thọ</t>
+          <t>Vo Van Tho</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bùi Đức Cường</t>
+          <t>Bui Duc Cuong</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Đinh Đức Tuấn</t>
+          <t>Dinh Duc Tuan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Trần Quang Thọ</t>
+          <t>Tran Quang Tho</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tô Hồng Giang</t>
+          <t>To Hong Giang</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vũ Minh Nghĩa</t>
+          <t>Vu Minh Nghia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Trần Hữu Mạnh</t>
+          <t>Tran Huu Manh</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hồ Đình Đạt</t>
+          <t>Ho Dinh Dat</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hồ Hồng Hạnh</t>
+          <t>Ho Hong Hanh</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hoàng Minh Tiến</t>
+          <t>Hoang Minh Tien</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -782,7 +782,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Đinh Thị Thảo</t>
+          <t>Dinh Thi Thao</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Huỳnh Đình An</t>
+          <t>Huynh Dinh An</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Đặng Quốc Sơn</t>
+          <t>Dang Quoc Son</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Phạm Hồng Yến</t>
+          <t>Pham Hong Yen</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lý Đức Thọ</t>
+          <t>Ly Duc Tho</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cao Xuân Vinh</t>
+          <t>Cao Xuan Vinh</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Đoàn Hồng Mai</t>
+          <t>Doan Hong Mai</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mai Quốc Hùng</t>
+          <t>Mai Quoc Hung</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Trần Hữu Cường</t>
+          <t>Tran Huu Cuong</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mai Tuấn Phong</t>
+          <t>Mai Tuan Phong</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Đỗ Xuân Nam</t>
+          <t>Do Xuan Nam</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bùi Đức Hùng</t>
+          <t>Bui Duc Hung</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Vũ Đức Nghĩa</t>
+          <t>Vu Duc Nghia</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Vũ Minh Nam</t>
+          <t>Vu Minh Nam</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hồ Mỹ Xuân</t>
+          <t>Ho My Xuan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Phan Văn Quý</t>
+          <t>Phan Van Quy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Trịnh Quốc Hải</t>
+          <t>Trinh Quoc Hai</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Đoàn Quang Mạnh</t>
+          <t>Doan Quang Manh</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mai Tuấn Phú</t>
+          <t>Mai Tuan Phu</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hoàng Thanh Nghĩa</t>
+          <t>Hoang Thanh Nghia</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Trịnh Thanh Đạt</t>
+          <t>Trinh Thanh Dat</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Đinh Thanh Sơn</t>
+          <t>Dinh Thanh Son</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hoàng Thanh Dũng</t>
+          <t>Hoang Thanh Dung</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Phan Thanh Phú</t>
+          <t>Phan Thanh Phu</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bùi Minh Tâm</t>
+          <t>Bui Minh Tam</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Trương Minh Quân</t>
+          <t>Truong Minh Quan</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Đặng Hồng Yến</t>
+          <t>Dang Hong Yen</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Đinh Xuân Sơn</t>
+          <t>Dinh Xuan Son</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Lâm Hồng Tuyết</t>
+          <t>Lam Hong Tuyet</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Lý Ngọc Hà</t>
+          <t>Ly Ngoc Ha</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Phan Xuân Long</t>
+          <t>Phan Xuan Long</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Phạm Mỹ Giang</t>
+          <t>Pham My Giang</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bùi Thu Quỳnh</t>
+          <t>Bui Thu Quynh</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Ngô Thị Ngân</t>
+          <t>Ngo Thi Ngan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Đoàn Hồng Quỳnh</t>
+          <t>Doan Hong Quynh</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Trương Mỹ Nhung</t>
+          <t>Truong My Nhung</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tạ Thị Hương</t>
+          <t>Ta Thi Huong</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Đoàn Ngọc Ngân</t>
+          <t>Doan Ngoc Ngan</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Hà Ngọc Thảo</t>
+          <t>Ha Ngoc Thao</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Cao Đức Nghĩa</t>
+          <t>Cao Duc Nghia</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Hoàng Thị Yến</t>
+          <t>Hoang Thi Yen</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Vũ Thanh Mai</t>
+          <t>Vu Thanh Mai</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Lâm Kim Ly</t>
+          <t>Lam Kim Ly</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Vũ Mỹ Trang</t>
+          <t>Vu My Trang</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Đặng Ngọc Hoa</t>
+          <t>Dang Ngoc Hoa</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Hoàng Quang Cường</t>
+          <t>Hoang Quang Cuong</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Ngô Xuân Trung</t>
+          <t>Ngo Xuan Trung</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Đặng Xuân Trí</t>
+          <t>Dang Xuan Tri</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ngô Diệu Anh</t>
+          <t>Ngo Dieu Anh</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Đinh Văn Tuấn</t>
+          <t>Dinh Van Tuan</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dương Minh Bích</t>
+          <t>Duong Minh Bich</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Hồ Mỹ Trang</t>
+          <t>Ho My Trang</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Đinh Thị Linh</t>
+          <t>Dinh Thi Linh</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Nguyễn Tuấn Đạt</t>
+          <t>Nguyen Tuan Dat</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Hà Hồng Giang</t>
+          <t>Ha Hong Giang</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Mai Xuân Mạnh</t>
+          <t>Mai Xuan Manh</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Đặng Tuấn Tiến</t>
+          <t>Dang Tuan Tien</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tô Hồng Anh</t>
+          <t>To Hong Anh</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Ngô Minh Thương</t>
+          <t>Ngo Minh Thuong</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Lâm Phương Hoa</t>
+          <t>Lam Phuong Hoa</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Mai Tuấn Thành</t>
+          <t>Mai Tuan Thanh</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Đỗ Thanh Long</t>
+          <t>Do Thanh Long</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Lâm Xuân Phong</t>
+          <t>Lam Xuan Phong</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Lê Mỹ Hạnh</t>
+          <t>Le My Hanh</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Đỗ Thu Thương</t>
+          <t>Do Thu Thuong</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Phạm Ngọc Lan</t>
+          <t>Pham Ngoc Lan</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Võ Tuấn Thọ</t>
+          <t>Vo Tuan Tho</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Huỳnh Mỹ Anh</t>
+          <t>Huynh My Anh</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Hoàng Diệu Diệp</t>
+          <t>Hoang Dieu Diep</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Trần Mỹ Vân</t>
+          <t>Tran My Van</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Thái Tuấn Vinh</t>
+          <t>Thai Tuan Vinh</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Hồ Đình Tuấn</t>
+          <t>Ho Dinh Tuan</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Nội Tim Mạch</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dương Tuấn Phong</t>
+          <t>Duong Tuan Phong</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Vũ Mỹ Tuyết</t>
+          <t>Vu My Tuyet</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Vũ Minh Xuân</t>
+          <t>Vu Minh Xuan</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Tạ Phương Xuân</t>
+          <t>Ta Phuong Xuan</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Trịnh Kim Nga</t>
+          <t>Trinh Kim Nga</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Hồi Sức Cấp Cứu</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Vũ Phương Phượng</t>
+          <t>Vu Phuong Phuong</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Dương Mỹ Giang</t>
+          <t>Duong My Giang</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Ngô Hữu Long</t>
+          <t>Ngo Huu Long</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Hồ Kim Bích</t>
+          <t>Ho Kim Bich</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Nội Tổng Quát</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Tạ Thị Thảo</t>
+          <t>Ta Thi Thao</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Sản</t>
+          <t>Obstetrics &amp; Gynecology</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Lý Diệu Trang</t>
+          <t>Ly Dieu Trang</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Nhi</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Lý Thanh Anh</t>
+          <t>Ly Thanh Anh</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Đinh Thu Chi</t>
+          <t>Dinh Thu Chi</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Ngoại Thần Kinh</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Đặng Kim Thúy</t>
+          <t>Dang Kim Thuy</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Chấn Thương Chỉnh Hình</t>
+          <t>Orthopedics</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Cao Quốc Thiện</t>
+          <t>Cao Quoc Thien</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Ung Bướu</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">

</xml_diff>